<commit_message>
updating the work report
</commit_message>
<xml_diff>
--- a/00_Docs/00_Work_Report/Ibrahim_Hegazi_Work_Report.xlsx
+++ b/00_Docs/00_Work_Report/Ibrahim_Hegazi_Work_Report.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14340" windowHeight="12435"/>
+    <workbookView windowWidth="14340" windowHeight="11910"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
   <si>
     <t>Project Name</t>
   </si>
@@ -130,7 +130,47 @@
     <t>Write the code that create the Unity Catalog and the needed Schemas in Databricks.</t>
   </si>
   <si>
+    <t>/01_Environment/01_Catalog_and_Schema_Creation.dbquery.ipynb</t>
+  </si>
+  <si>
     <t>Write the code that gives you all the privileges on the catalog, schemas, and volumes that you created in the previous step.</t>
+  </si>
+  <si>
+    <t>/01_Environment/02_GRANT_PRIVILEGES.dbquery.ipynb</t>
+  </si>
+  <si>
+    <t>Create the .env and .gitignore files so that you can add kaggle dataset API key there safely</t>
+  </si>
+  <si>
+    <t>Extract the data from kaggle from https://www.kaggle.com/datasets/yelp-dataset/yelp-dataset/data</t>
+  </si>
+  <si>
+    <t>Now that the initial Environment is ready, we can extract the data now.</t>
+  </si>
+  <si>
+    <t>The dataset size is big and needs the companies internet.</t>
+  </si>
+  <si>
+    <t>Not going back home till I get sure that the dataset can be downloaded from databricks' servers internet or the company's internet.</t>
+  </si>
+  <si>
+    <t>Downlaod the Yelp Images from https://business.yelp.com/data/resources/open-dataset/ because kaggle only contains the textual data ( 25 minutes needed using the companies internet )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The data extracted form kaggle was not complete and the images was not download.
+</t>
+  </si>
+  <si>
+    <t>Manually download the data on my device locally then i will upload it on databricks volume.</t>
+  </si>
+  <si>
+    <t>Completed But the pipeline is not idempotent at the time being after you finish you Profiling, EDA, Bronze, Silver, Gold, you will need to search about yelp API to see if you download this dataset automatically</t>
+  </si>
+  <si>
+    <t>Upload the images from your local device to databricks</t>
+  </si>
+  <si>
+    <t>THE REAL ISSUE: The compressed file is bigger than databricks upload limit in terms of the over all size and the upcompressed version contains alot of files in terms of their number and it is greater than databricks upload limit in terms of the number of files to uploaded.</t>
   </si>
   <si>
     <t>Study and Understand Service Principle so that the work that your account does don't go to waste if the account got deleted.</t>
@@ -148,9 +188,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -198,6 +238,37 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -214,7 +285,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -222,21 +293,21 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -252,45 +323,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -305,21 +338,28 @@
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
@@ -336,49 +376,151 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -390,13 +532,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -408,55 +544,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -468,55 +556,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -527,6 +567,39 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -562,15 +635,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -595,21 +659,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -618,156 +667,147 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
@@ -1525,11 +1565,14 @@
       <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="J5" s="1" t="s">
+        <v>37</v>
+      </c>
       <c r="L5" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1" spans="1:5">
+    <row r="6" ht="45" customHeight="1" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1537,7 +1580,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>15</v>
@@ -1545,8 +1588,14 @@
       <c r="E6" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" ht="75" customHeight="1" spans="1:5">
+      <c r="J6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" ht="45" spans="1:12">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1554,16 +1603,19 @@
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1" spans="1:5">
+        <v>15</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1" spans="1:8">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1571,24 +1623,102 @@
         <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" ht="90" customHeight="1" spans="2:2">
-      <c r="B9" s="5"/>
-    </row>
-    <row r="10" ht="60" customHeight="1"/>
+        <v>15</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" spans="1:12">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1" spans="1:7">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="11" ht="75" customHeight="1"/>
-    <row r="12" ht="60" customHeight="1" spans="2:2">
-      <c r="B12" s="5"/>
-    </row>
-    <row r="13" ht="75" customHeight="1"/>
+    <row r="12" ht="60" customHeight="1" spans="1:5">
+      <c r="A12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1" spans="1:5">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
     <row r="14" ht="120" customHeight="1"/>
     <row r="15" ht="105" customHeight="1"/>
     <row r="16" ht="60" customHeight="1" spans="2:2">

</xml_diff>